<commit_message>
Apply green brand color scheme to workbook
Recolor headers, titles, and alternating row shading from navy to
brand green across the combined sheet and all 21 Regional Center tabs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfUqFbprquvj5oFM5dTRgv
</commit_message>
<xml_diff>
--- a/FMS_Contact_List_and_Employer_Burden.xlsx
+++ b/FMS_Contact_List_and_Employer_Burden.xlsx
@@ -71,7 +71,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000B3D62"/>
+      <color rgb="001B7A3D"/>
       <sz val="14"/>
     </font>
     <font>
@@ -97,12 +97,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B3D62"/>
+        <fgColor rgb="001B7A3D"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F6FA"/>
+        <fgColor rgb="00EAF4EC"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>